<commit_message>
MR24-038: Day 3 (808 down)
</commit_message>
<xml_diff>
--- a/data/mr24-038-experiment/MR24-038-MasterDataTable.xlsx
+++ b/data/mr24-038-experiment/MR24-038-MasterDataTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/MR24-038-MPC-3L/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="360" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42306D88-6FD8-4A84-93C1-C28BC91718EC}"/>
+  <xr:revisionPtr revIDLastSave="422" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5D559AA-9825-4149-9AC4-E308E382366B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MasterDataTable!$A$2:$BM$277</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,8 +39,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={FF16B357-339F-45F1-8E08-77BC469B5CFA}</author>
+  </authors>
+  <commentList>
+    <comment ref="BI12" authorId="0" shapeId="0" xr:uid="{FF16B357-339F-45F1-8E08-77BC469B5CFA}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Override MPC feed rate with CSFR</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="84">
   <si>
     <t>Batch Data</t>
   </si>
@@ -284,6 +301,15 @@
   </si>
   <si>
     <t>Reactor was found to be contaminated</t>
+  </si>
+  <si>
+    <t>Changed to CSFR flow rate until Julia code was run at 4pm</t>
+  </si>
+  <si>
+    <t>CSFR Flow rates were used</t>
+  </si>
+  <si>
+    <t>Contaminated on day 3</t>
   </si>
 </sst>
 </file>
@@ -966,7 +992,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -1049,6 +1075,17 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="41" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="14" fillId="38" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1100,10 +1137,6 @@
     <xf numFmtId="0" fontId="19" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1192,6 +1225,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Yu Luo" id="{39B0911F-58E9-4732-93E1-F7F715DFAAAC}" userId="S::yu.8.luo@gsk.com::5e93f0cf-7e56-492e-afc9-2cfd7b5fd269" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1489,13 +1528,22 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="BI12" dT="2024-07-20T18:22:09.75" personId="{39B0911F-58E9-4732-93E1-F7F715DFAAAC}" id="{FF16B357-339F-45F1-8E08-77BC469B5CFA}">
+    <text>Override MPC feed rate with CSFR</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:BP46"/>
   <sheetFormatPr defaultColWidth="14.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="5" width="10.6640625" customWidth="1"/>
+    <col min="2" max="4" width="10.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.88671875" customWidth="1"/>
     <col min="6" max="6" width="16.88671875" customWidth="1"/>
     <col min="7" max="18" width="12.6640625" customWidth="1"/>
     <col min="19" max="19" width="15.109375" bestFit="1" customWidth="1"/>
@@ -1506,88 +1554,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:68" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="66" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
-      <c r="G1" s="67" t="s">
+      <c r="A1" s="75" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
-      <c r="AC1" s="68"/>
-      <c r="AD1" s="69"/>
-      <c r="AE1" s="80" t="s">
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
+      <c r="O1" s="77"/>
+      <c r="P1" s="77"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="77"/>
+      <c r="W1" s="77"/>
+      <c r="X1" s="77"/>
+      <c r="Y1" s="77"/>
+      <c r="Z1" s="77"/>
+      <c r="AA1" s="77"/>
+      <c r="AB1" s="77"/>
+      <c r="AC1" s="77"/>
+      <c r="AD1" s="78"/>
+      <c r="AE1" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="AF1" s="81"/>
-      <c r="AG1" s="81"/>
-      <c r="AH1" s="81"/>
-      <c r="AI1" s="81"/>
-      <c r="AJ1" s="81"/>
-      <c r="AK1" s="81"/>
-      <c r="AL1" s="81"/>
-      <c r="AM1" s="81"/>
-      <c r="AN1" s="81"/>
-      <c r="AO1" s="81"/>
-      <c r="AP1" s="81"/>
-      <c r="AQ1" s="81"/>
-      <c r="AR1" s="81"/>
-      <c r="AS1" s="81"/>
-      <c r="AT1" s="82"/>
-      <c r="AU1" s="75" t="s">
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="90"/>
+      <c r="AH1" s="90"/>
+      <c r="AI1" s="90"/>
+      <c r="AJ1" s="90"/>
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="90"/>
+      <c r="AP1" s="90"/>
+      <c r="AQ1" s="90"/>
+      <c r="AR1" s="90"/>
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="91"/>
+      <c r="AU1" s="84" t="s">
         <v>3</v>
       </c>
-      <c r="AV1" s="75"/>
-      <c r="AW1" s="75"/>
-      <c r="AX1" s="75"/>
-      <c r="AY1" s="76"/>
-      <c r="AZ1" s="77" t="s">
+      <c r="AV1" s="84"/>
+      <c r="AW1" s="84"/>
+      <c r="AX1" s="84"/>
+      <c r="AY1" s="85"/>
+      <c r="AZ1" s="86" t="s">
         <v>4</v>
       </c>
-      <c r="BA1" s="78"/>
-      <c r="BB1" s="79"/>
-      <c r="BC1" s="73" t="s">
+      <c r="BA1" s="87"/>
+      <c r="BB1" s="88"/>
+      <c r="BC1" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="BD1" s="74"/>
-      <c r="BE1" s="74"/>
-      <c r="BF1" s="74"/>
-      <c r="BG1" s="74"/>
-      <c r="BH1" s="74"/>
-      <c r="BI1" s="74"/>
-      <c r="BJ1" s="74"/>
-      <c r="BK1" s="74"/>
-      <c r="BL1" s="74"/>
-      <c r="BM1" s="74"/>
-      <c r="BN1" s="70" t="s">
+      <c r="BD1" s="83"/>
+      <c r="BE1" s="83"/>
+      <c r="BF1" s="83"/>
+      <c r="BG1" s="83"/>
+      <c r="BH1" s="83"/>
+      <c r="BI1" s="83"/>
+      <c r="BJ1" s="83"/>
+      <c r="BK1" s="83"/>
+      <c r="BL1" s="83"/>
+      <c r="BM1" s="83"/>
+      <c r="BN1" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="BO1" s="71"/>
-      <c r="BP1" s="72"/>
+      <c r="BO1" s="80"/>
+      <c r="BP1" s="81"/>
     </row>
     <row r="2" spans="1:68" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
@@ -1602,7 +1650,7 @@
       <c r="D2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="E2" s="72" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="26" t="s">
@@ -1809,7 +1857,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="84">
+      <c r="F3" s="66">
         <v>45491.472488425898</v>
       </c>
       <c r="G3" s="3">
@@ -2010,17 +2058,16 @@
       <c r="A4" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="83" t="s">
+      <c r="B4" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="83">
+      <c r="C4">
         <v>12</v>
       </c>
-      <c r="D4" s="83">
-        <v>0</v>
-      </c>
-      <c r="E4" s="83"/>
-      <c r="F4" s="85">
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="67">
         <v>45491.474918981497</v>
       </c>
       <c r="G4">
@@ -2221,17 +2268,16 @@
       <c r="A5" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B5" s="83" t="s">
+      <c r="B5" t="s">
         <v>78</v>
       </c>
-      <c r="C5" s="83">
+      <c r="C5">
         <v>12</v>
       </c>
-      <c r="D5" s="83">
-        <v>0</v>
-      </c>
-      <c r="E5" s="83"/>
-      <c r="F5" s="85">
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="F5" s="67">
         <v>45491.477488425902</v>
       </c>
       <c r="G5">
@@ -2441,7 +2487,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="5"/>
-      <c r="F6" s="86">
+      <c r="F6" s="68">
         <v>45491.480787036999</v>
       </c>
       <c r="G6" s="5">
@@ -2652,7 +2698,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="85">
+      <c r="F7" s="67">
         <v>45492.338194444441</v>
       </c>
       <c r="G7" s="3">
@@ -2859,19 +2905,19 @@
       <c r="A8" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B8" s="83" t="s">
+      <c r="B8" t="s">
         <v>75</v>
       </c>
-      <c r="C8" s="83">
+      <c r="C8">
         <v>12</v>
       </c>
-      <c r="D8" s="83">
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" s="83" t="s">
+      <c r="E8" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="85">
+      <c r="F8" s="67">
         <v>45492.34097222222</v>
       </c>
       <c r="G8">
@@ -3078,17 +3124,16 @@
       <c r="A9" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="83" t="s">
+      <c r="B9" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="83">
+      <c r="C9">
         <v>12</v>
       </c>
-      <c r="D9" s="83">
+      <c r="D9">
         <v>1</v>
       </c>
-      <c r="E9" s="83"/>
-      <c r="F9" s="85">
+      <c r="F9" s="67">
         <v>45492.34375</v>
       </c>
       <c r="G9">
@@ -3291,17 +3336,16 @@
       <c r="A10" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="83" t="s">
+      <c r="B10" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="83">
+      <c r="C10">
         <v>12</v>
       </c>
-      <c r="D10" s="83">
+      <c r="D10">
         <v>1</v>
       </c>
-      <c r="E10" s="83"/>
-      <c r="F10" s="85">
+      <c r="F10" s="67">
         <v>45492.345833333333</v>
       </c>
       <c r="G10" s="5">
@@ -3515,8 +3559,10 @@
       <c r="D11" s="3">
         <v>2</v>
       </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="84">
+      <c r="E11" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="66">
         <v>45493.525694444397</v>
       </c>
       <c r="G11">
@@ -3614,7 +3660,7 @@
       </c>
       <c r="AM11" s="56">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1.9587601193460299E-2</v>
       </c>
       <c r="AN11" s="6">
         <v>16</v>
@@ -3656,9 +3702,15 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="AZ11" s="8"/>
-      <c r="BA11" s="9"/>
-      <c r="BB11" s="28"/>
-      <c r="BC11" s="8">
+      <c r="BA11" s="9">
+        <f>BJ11*24*60/BE11</f>
+        <v>1.6416168450565701E-2</v>
+      </c>
+      <c r="BB11" s="28">
+        <f>BM11/BE11</f>
+        <v>7.0438155546433375E-3</v>
+      </c>
+      <c r="BC11" s="71">
         <f t="shared" si="0"/>
         <v>1.1494711169999998E-2</v>
       </c>
@@ -3680,15 +3732,14 @@
       </c>
       <c r="BH11" s="10">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>28.206145718582832</v>
       </c>
       <c r="BI11" s="10" t="str">
-        <f t="shared" si="10"/>
+        <f>IF(B11="Python",AZ11*BE11/24/60,"")</f>
         <v/>
       </c>
       <c r="BJ11" s="10">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <v>1.9587601193460299E-2</v>
       </c>
       <c r="BK11" s="45" t="str">
         <f t="shared" si="6"/>
@@ -3699,37 +3750,38 @@
         <v/>
       </c>
       <c r="BM11" s="10">
-        <f t="shared" si="14"/>
-        <v>0</v>
+        <v>12.1026345792793</v>
       </c>
       <c r="BN11" s="34">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>50.876886216780001</v>
       </c>
       <c r="BO11" s="48">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1.9587601193460299E-2</v>
       </c>
       <c r="BP11" s="39">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>12.1026345792793</v>
       </c>
     </row>
     <row r="12" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="83" t="s">
+      <c r="B12" t="s">
         <v>78</v>
       </c>
-      <c r="C12" s="83">
+      <c r="C12">
         <v>12</v>
       </c>
-      <c r="D12" s="83">
+      <c r="D12">
         <v>2</v>
       </c>
-      <c r="E12" s="83"/>
-      <c r="F12" s="85">
+      <c r="E12" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="67">
         <v>45493.528472222199</v>
       </c>
       <c r="G12">
@@ -3827,7 +3879,7 @@
       </c>
       <c r="AM12" s="57">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1.190824173E-2</v>
       </c>
       <c r="AN12" s="22">
         <v>16</v>
@@ -3868,9 +3920,11 @@
       <c r="AY12" s="23">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="AZ12" s="11"/>
+      <c r="AZ12" s="11">
+        <v>4.4999999999999997E-3</v>
+      </c>
       <c r="BB12" s="29"/>
-      <c r="BC12" s="11">
+      <c r="BC12" s="69">
         <f t="shared" si="0"/>
         <v>1.190824173E-2</v>
       </c>
@@ -3892,11 +3946,10 @@
       </c>
       <c r="BH12" s="24">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="BI12" s="24">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <v>17.147868091199999</v>
+      </c>
+      <c r="BI12" s="73">
+        <v>1.190824173E-2</v>
       </c>
       <c r="BJ12" s="24" t="str">
         <f t="shared" si="13"/>
@@ -3916,11 +3969,11 @@
       </c>
       <c r="BN12" s="35">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>30.930498</v>
       </c>
       <c r="BO12" s="49">
-        <f t="shared" si="12"/>
-        <v>0</v>
+        <f>IF(BI12&lt;&gt;"",BI12,IF(BJ12&lt;&gt;"",BJ12,BK12))</f>
+        <v>1.190824173E-2</v>
       </c>
       <c r="BP12" s="37">
         <f t="shared" si="7"/>
@@ -3940,8 +3993,10 @@
       <c r="D13" s="5">
         <v>2</v>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="86">
+      <c r="E13" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F13" s="68">
         <v>45493.536805555603</v>
       </c>
       <c r="G13">
@@ -4039,7 +4094,7 @@
       </c>
       <c r="AM13" s="58">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1.1710864169999998E-2</v>
       </c>
       <c r="AN13" s="7">
         <v>18</v>
@@ -4080,9 +4135,11 @@
       <c r="AY13" s="13">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="AZ13" s="12"/>
+      <c r="AZ13" s="12">
+        <v>4.5000000009706104E-3</v>
+      </c>
       <c r="BB13" s="30"/>
-      <c r="BC13" s="12">
+      <c r="BC13" s="70">
         <f t="shared" si="0"/>
         <v>1.1710864169999998E-2</v>
       </c>
@@ -4104,11 +4161,10 @@
       </c>
       <c r="BH13" s="14">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="BI13" s="14">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <v>16.863644404799995</v>
+      </c>
+      <c r="BI13" s="74">
+        <v>1.1710864169999998E-2</v>
       </c>
       <c r="BJ13" s="14" t="str">
         <f t="shared" si="13"/>
@@ -4128,11 +4184,11 @@
       </c>
       <c r="BN13" s="36">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>30.41782901298701</v>
       </c>
       <c r="BO13" s="50">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1.1710864169999998E-2</v>
       </c>
       <c r="BP13" s="38">
         <f t="shared" si="7"/>
@@ -4153,62 +4209,126 @@
         <v>3</v>
       </c>
       <c r="E14" s="3"/>
-      <c r="F14" s="84"/>
+      <c r="F14" s="66">
+        <v>45494.550289351901</v>
+      </c>
       <c r="G14" s="3">
         <v>1505.08</v>
       </c>
       <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
+      <c r="I14" s="6">
+        <v>1446.18</v>
+      </c>
+      <c r="J14" s="6">
+        <v>24</v>
+      </c>
+      <c r="K14" s="6">
+        <v>23.1</v>
+      </c>
+      <c r="L14" s="6">
+        <v>96</v>
+      </c>
+      <c r="M14" s="6">
+        <v>17.100000000000001</v>
+      </c>
+      <c r="N14" s="6">
+        <v>350</v>
+      </c>
+      <c r="O14" s="6">
+        <v>1.58</v>
+      </c>
+      <c r="P14" s="6">
+        <v>0.38</v>
+      </c>
+      <c r="Q14" s="6">
+        <v>2.0099999999999998</v>
+      </c>
       <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
-      <c r="V14" s="6"/>
-      <c r="W14" s="6"/>
-      <c r="X14" s="6"/>
-      <c r="Y14" s="6"/>
-      <c r="Z14" s="6"/>
-      <c r="AA14" s="6"/>
-      <c r="AB14" s="6"/>
-      <c r="AC14" s="6"/>
-      <c r="AD14" s="19"/>
-      <c r="AE14" s="53"/>
-      <c r="AF14" s="6"/>
-      <c r="AG14" s="6"/>
+      <c r="S14" s="6">
+        <v>0</v>
+      </c>
+      <c r="T14" s="6">
+        <v>0.03</v>
+      </c>
+      <c r="U14" s="6">
+        <v>2.76</v>
+      </c>
+      <c r="V14" s="6">
+        <v>7.218</v>
+      </c>
+      <c r="W14" s="6">
+        <v>139.80000000000001</v>
+      </c>
+      <c r="X14" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="6">
+        <v>2.92</v>
+      </c>
+      <c r="Z14" s="6">
+        <v>149</v>
+      </c>
+      <c r="AA14" s="6">
+        <v>55.4</v>
+      </c>
+      <c r="AB14" s="6">
+        <v>122.6</v>
+      </c>
+      <c r="AC14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AD14" s="19">
+        <v>7.2590000000000003</v>
+      </c>
+      <c r="AE14" s="53">
+        <v>300</v>
+      </c>
+      <c r="AF14" s="6">
+        <v>49.2</v>
+      </c>
+      <c r="AG14" s="6">
+        <v>7.19</v>
+      </c>
       <c r="AH14" s="56">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="AI14" s="6"/>
-      <c r="AJ14" s="6"/>
-      <c r="AK14" s="6"/>
-      <c r="AL14" s="6"/>
+        <v>0.49200000000000005</v>
+      </c>
+      <c r="AI14" s="6">
+        <v>34</v>
+      </c>
+      <c r="AJ14" s="6">
+        <v>27.664999999999999</v>
+      </c>
+      <c r="AK14" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL14" s="6">
+        <v>4</v>
+      </c>
       <c r="AM14" s="56">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AN14" s="6"/>
-      <c r="AO14" s="6"/>
-      <c r="AP14" s="6"/>
+      <c r="AN14" s="6">
+        <v>42</v>
+      </c>
+      <c r="AO14" s="6">
+        <v>31</v>
+      </c>
+      <c r="AP14" s="6">
+        <v>668</v>
+      </c>
       <c r="AQ14" s="56">
         <f t="shared" si="20"/>
-        <v>-16</v>
+        <v>26</v>
       </c>
       <c r="AR14" s="56">
         <f t="shared" si="21"/>
-        <v>-18</v>
+        <v>13</v>
       </c>
       <c r="AS14" s="56">
         <f t="shared" si="22"/>
-        <v>695</v>
+        <v>27</v>
       </c>
       <c r="AT14" s="31">
         <v>15</v>
@@ -4233,23 +4353,23 @@
       <c r="BB14" s="28"/>
       <c r="BC14" s="8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.2090528449999999E-2</v>
       </c>
       <c r="BD14" s="9">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>17.410360967999999</v>
       </c>
       <c r="BE14" s="9">
         <f t="shared" si="17"/>
-        <v>1640</v>
-      </c>
-      <c r="BF14" s="10" t="e">
+        <v>1744.665</v>
+      </c>
+      <c r="BF14" s="10">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="BG14" s="10" t="e">
+        <v>2.4073389447257783E-2</v>
+      </c>
+      <c r="BG14" s="10">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
+        <v>2.4705882352941175E-2</v>
       </c>
       <c r="BH14" s="10">
         <f t="shared" si="5"/>
@@ -4292,72 +4412,135 @@
       <c r="A15" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="83" t="s">
+      <c r="B15" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="83">
+      <c r="C15">
         <v>12</v>
       </c>
-      <c r="D15" s="83">
+      <c r="D15">
         <v>3</v>
       </c>
-      <c r="E15" s="83"/>
-      <c r="F15" s="85"/>
+      <c r="F15" s="67">
+        <v>45494.554664351897</v>
+      </c>
       <c r="G15">
         <v>1505.08</v>
       </c>
       <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
+      <c r="I15" s="22">
+        <v>1350.49</v>
+      </c>
+      <c r="J15" s="22">
+        <v>24</v>
+      </c>
+      <c r="K15" s="22">
+        <v>22.7</v>
+      </c>
+      <c r="L15" s="22">
+        <v>94.4</v>
+      </c>
+      <c r="M15" s="22">
+        <v>16.5</v>
+      </c>
+      <c r="N15" s="22">
+        <v>372</v>
+      </c>
+      <c r="O15" s="22">
+        <v>2.68</v>
+      </c>
+      <c r="P15" s="22">
+        <v>0.4</v>
+      </c>
+      <c r="Q15" s="22">
+        <v>0.01</v>
+      </c>
       <c r="R15" s="22"/>
-      <c r="S15" s="22"/>
-      <c r="T15" s="22"/>
-      <c r="U15" s="22"/>
-      <c r="V15" s="22"/>
-      <c r="W15" s="22"/>
-      <c r="X15" s="22"/>
-      <c r="Y15" s="22"/>
-      <c r="Z15" s="22"/>
-      <c r="AA15" s="22"/>
-      <c r="AB15" s="22"/>
-      <c r="AC15" s="22"/>
-      <c r="AD15" s="20"/>
-      <c r="AE15" s="54"/>
-      <c r="AF15" s="22"/>
-      <c r="AG15" s="22"/>
+      <c r="S15" s="22">
+        <v>0.08</v>
+      </c>
+      <c r="T15" s="22">
+        <v>0.1</v>
+      </c>
+      <c r="U15" s="22">
+        <v>3.17</v>
+      </c>
+      <c r="V15" s="22">
+        <v>7.3440000000000003</v>
+      </c>
+      <c r="W15" s="22">
+        <v>146.69999999999999</v>
+      </c>
+      <c r="X15" s="22">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="22">
+        <v>3.6</v>
+      </c>
+      <c r="Z15" s="22">
+        <v>167.8</v>
+      </c>
+      <c r="AA15" s="22">
+        <v>78</v>
+      </c>
+      <c r="AB15" s="22">
+        <v>128.6</v>
+      </c>
+      <c r="AC15" s="22">
+        <v>0</v>
+      </c>
+      <c r="AD15" s="20">
+        <v>7.3869999999999996</v>
+      </c>
+      <c r="AE15" s="54">
+        <v>300</v>
+      </c>
+      <c r="AF15" s="22">
+        <v>52.2</v>
+      </c>
+      <c r="AG15" s="22">
+        <v>7.29</v>
+      </c>
       <c r="AH15" s="57">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="AI15" s="22"/>
-      <c r="AJ15" s="22"/>
-      <c r="AK15" s="22"/>
-      <c r="AL15" s="22"/>
+        <v>0.52200000000000002</v>
+      </c>
+      <c r="AI15" s="22">
+        <v>34</v>
+      </c>
+      <c r="AJ15" s="22">
+        <v>37.567</v>
+      </c>
+      <c r="AK15" s="22">
+        <v>0</v>
+      </c>
+      <c r="AL15" s="22">
+        <v>4</v>
+      </c>
       <c r="AM15" s="57">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AN15" s="22"/>
-      <c r="AO15" s="22"/>
-      <c r="AP15" s="22"/>
+      <c r="AN15" s="22">
+        <v>33</v>
+      </c>
+      <c r="AO15" s="22">
+        <v>34</v>
+      </c>
+      <c r="AP15" s="22">
+        <v>743</v>
+      </c>
       <c r="AQ15" s="57">
         <f t="shared" si="20"/>
-        <v>-16</v>
+        <v>17</v>
       </c>
       <c r="AR15" s="57">
         <f t="shared" si="21"/>
-        <v>-20</v>
+        <v>14</v>
       </c>
       <c r="AS15" s="57">
         <f t="shared" si="22"/>
-        <v>762</v>
+        <v>19</v>
       </c>
       <c r="AT15" s="32">
         <v>15</v>
@@ -4382,23 +4565,23 @@
       <c r="BB15" s="29"/>
       <c r="BC15" s="11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.1907741269999999E-2</v>
       </c>
       <c r="BD15" s="23">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>17.147147428799997</v>
       </c>
       <c r="BE15" s="23">
         <f t="shared" si="17"/>
-        <v>1640</v>
-      </c>
-      <c r="BF15" s="24" t="e">
+        <v>1748.567</v>
+      </c>
+      <c r="BF15" s="24">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="BG15" s="24" t="e">
+        <v>1.8872596817851417E-2</v>
+      </c>
+      <c r="BG15" s="24">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
+        <v>1.9411764705882354E-2</v>
       </c>
       <c r="BH15" s="24">
         <f t="shared" si="5"/>
@@ -4418,7 +4601,7 @@
       </c>
       <c r="BL15" s="24">
         <f t="shared" si="19"/>
-        <v>12.3</v>
+        <v>13.070538324999999</v>
       </c>
       <c r="BM15" s="24" t="str">
         <f t="shared" si="14"/>
@@ -4434,7 +4617,7 @@
       </c>
       <c r="BP15" s="37">
         <f t="shared" si="7"/>
-        <v>12.3</v>
+        <v>13.070538324999999</v>
       </c>
     </row>
     <row r="16" spans="1:68" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -4450,8 +4633,10 @@
       <c r="D16" s="5">
         <v>3</v>
       </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="86"/>
+      <c r="E16" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="68"/>
       <c r="G16" s="5">
         <v>1505.08</v>
       </c>
@@ -4478,35 +4663,55 @@
       <c r="AB16" s="7"/>
       <c r="AC16" s="7"/>
       <c r="AD16" s="21"/>
-      <c r="AE16" s="55"/>
-      <c r="AF16" s="7"/>
-      <c r="AG16" s="7"/>
+      <c r="AE16" s="55">
+        <v>300</v>
+      </c>
+      <c r="AF16" s="7">
+        <v>11.1</v>
+      </c>
+      <c r="AG16" s="7">
+        <v>7.31</v>
+      </c>
       <c r="AH16" s="58">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="AI16" s="7"/>
-      <c r="AJ16" s="7"/>
-      <c r="AK16" s="7"/>
-      <c r="AL16" s="7"/>
+        <v>0.111</v>
+      </c>
+      <c r="AI16" s="7">
+        <v>34</v>
+      </c>
+      <c r="AJ16" s="7">
+        <v>38.723999999999997</v>
+      </c>
+      <c r="AK16" s="7">
+        <v>8.9086999999999996</v>
+      </c>
+      <c r="AL16" s="7">
+        <v>3</v>
+      </c>
       <c r="AM16" s="58">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AN16" s="7"/>
-      <c r="AO16" s="7"/>
-      <c r="AP16" s="7"/>
+      <c r="AN16" s="7">
+        <v>34</v>
+      </c>
+      <c r="AO16" s="7">
+        <v>30</v>
+      </c>
+      <c r="AP16" s="7">
+        <v>591</v>
+      </c>
       <c r="AQ16" s="58">
         <f t="shared" si="20"/>
-        <v>-18</v>
+        <v>16</v>
       </c>
       <c r="AR16" s="58">
         <f t="shared" si="21"/>
-        <v>-18</v>
+        <v>12</v>
       </c>
       <c r="AS16" s="58">
         <f t="shared" si="22"/>
-        <v>608</v>
+        <v>17</v>
       </c>
       <c r="AT16" s="33">
         <v>15</v>
@@ -4539,15 +4744,15 @@
       </c>
       <c r="BE16" s="13">
         <f t="shared" si="17"/>
-        <v>1640</v>
-      </c>
-      <c r="BF16" s="14" t="e">
+        <v>1754.6327000000001</v>
+      </c>
+      <c r="BF16" s="14">
         <f t="shared" si="3"/>
-        <v>#N/A</v>
-      </c>
-      <c r="BG16" s="14" t="e">
+        <v>1.9377274799449479E-2</v>
+      </c>
+      <c r="BG16" s="14">
         <f t="shared" si="4"/>
-        <v>#N/A</v>
+        <v>0.02</v>
       </c>
       <c r="BH16" s="14">
         <f t="shared" si="5"/>
@@ -4567,7 +4772,7 @@
       </c>
       <c r="BL16" s="14">
         <f t="shared" si="19"/>
-        <v>12.3</v>
+        <v>13.15974525</v>
       </c>
       <c r="BM16" s="14" t="str">
         <f t="shared" si="14"/>
@@ -4583,24 +4788,23 @@
       </c>
       <c r="BP16" s="37">
         <f t="shared" si="7"/>
-        <v>12.3</v>
+        <v>13.15974525</v>
       </c>
     </row>
     <row r="17" spans="1:68" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B17" s="83" t="s">
+      <c r="B17" t="s">
         <v>75</v>
       </c>
-      <c r="C17" s="83">
+      <c r="C17">
         <v>12</v>
       </c>
-      <c r="D17" s="83">
+      <c r="D17">
         <v>4</v>
       </c>
-      <c r="E17" s="83"/>
-      <c r="F17" s="85"/>
+      <c r="F17" s="67"/>
       <c r="G17">
         <v>2119.61</v>
       </c>
@@ -4647,15 +4851,15 @@
       <c r="AP17" s="6"/>
       <c r="AQ17" s="56">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-42</v>
       </c>
       <c r="AR17" s="56">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>-31</v>
       </c>
       <c r="AS17" s="56">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>668</v>
       </c>
       <c r="AT17" s="31">
         <v>15</v>
@@ -4739,17 +4943,16 @@
       <c r="A18" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="83" t="s">
+      <c r="B18" t="s">
         <v>78</v>
       </c>
-      <c r="C18" s="83">
+      <c r="C18">
         <v>12</v>
       </c>
-      <c r="D18" s="83">
+      <c r="D18">
         <v>4</v>
       </c>
-      <c r="E18" s="83"/>
-      <c r="F18" s="85"/>
+      <c r="F18" s="67"/>
       <c r="G18">
         <v>2119.61</v>
       </c>
@@ -4796,15 +4999,15 @@
       <c r="AP18" s="22"/>
       <c r="AQ18" s="57">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-33</v>
       </c>
       <c r="AR18" s="57">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>-34</v>
       </c>
       <c r="AS18" s="57">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>743</v>
       </c>
       <c r="AT18" s="32">
         <v>15</v>
@@ -4888,17 +5091,16 @@
       <c r="A19" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="83" t="s">
+      <c r="B19" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="83">
+      <c r="C19">
         <v>12</v>
       </c>
-      <c r="D19" s="83">
+      <c r="D19">
         <v>4</v>
       </c>
-      <c r="E19" s="83"/>
-      <c r="F19" s="85"/>
+      <c r="F19" s="67"/>
       <c r="G19">
         <v>2119.61</v>
       </c>
@@ -4945,15 +5147,15 @@
       <c r="AP19" s="7"/>
       <c r="AQ19" s="58">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>-34</v>
       </c>
       <c r="AR19" s="58">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>-30</v>
       </c>
       <c r="AS19" s="58">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>591</v>
       </c>
       <c r="AT19" s="33">
         <v>15</v>
@@ -5047,7 +5249,7 @@
         <v>5</v>
       </c>
       <c r="E20" s="3"/>
-      <c r="F20" s="84"/>
+      <c r="F20" s="66"/>
       <c r="G20" s="3">
         <v>2716.05</v>
       </c>
@@ -5186,17 +5388,16 @@
       <c r="A21" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="83" t="s">
+      <c r="B21" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="83">
+      <c r="C21">
         <v>12</v>
       </c>
-      <c r="D21" s="83">
+      <c r="D21">
         <v>5</v>
       </c>
-      <c r="E21" s="83"/>
-      <c r="F21" s="85"/>
+      <c r="F21" s="67"/>
       <c r="G21">
         <v>2716.05</v>
       </c>
@@ -5345,7 +5546,7 @@
         <v>5</v>
       </c>
       <c r="E22" s="5"/>
-      <c r="F22" s="86"/>
+      <c r="F22" s="68"/>
       <c r="G22" s="5">
         <v>2716.05</v>
       </c>
@@ -5484,17 +5685,16 @@
       <c r="A23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="83" t="s">
+      <c r="B23" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="83">
+      <c r="C23">
         <v>12</v>
       </c>
-      <c r="D23" s="83">
+      <c r="D23">
         <v>6</v>
       </c>
-      <c r="E23" s="83"/>
-      <c r="F23" s="85"/>
+      <c r="F23" s="67"/>
       <c r="G23">
         <v>3307.9</v>
       </c>
@@ -5633,17 +5833,16 @@
       <c r="A24" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B24" s="83" t="s">
+      <c r="B24" t="s">
         <v>78</v>
       </c>
-      <c r="C24" s="83">
+      <c r="C24">
         <v>12</v>
       </c>
-      <c r="D24" s="83">
+      <c r="D24">
         <v>6</v>
       </c>
-      <c r="E24" s="83"/>
-      <c r="F24" s="85"/>
+      <c r="F24" s="67"/>
       <c r="G24">
         <v>3307.9</v>
       </c>
@@ -5782,17 +5981,16 @@
       <c r="A25" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="83" t="s">
+      <c r="B25" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="83">
+      <c r="C25">
         <v>12</v>
       </c>
-      <c r="D25" s="83">
+      <c r="D25">
         <v>6</v>
       </c>
-      <c r="E25" s="83"/>
-      <c r="F25" s="85"/>
+      <c r="F25" s="67"/>
       <c r="G25">
         <v>3307.9</v>
       </c>
@@ -5941,7 +6139,7 @@
         <v>7</v>
       </c>
       <c r="E26" s="3"/>
-      <c r="F26" s="84"/>
+      <c r="F26" s="66"/>
       <c r="G26" s="3">
         <v>3888.32</v>
       </c>
@@ -6080,17 +6278,16 @@
       <c r="A27" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B27" s="83" t="s">
+      <c r="B27" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="83">
+      <c r="C27">
         <v>12</v>
       </c>
-      <c r="D27" s="83">
+      <c r="D27">
         <v>7</v>
       </c>
-      <c r="E27" s="83"/>
-      <c r="F27" s="85"/>
+      <c r="F27" s="67"/>
       <c r="G27">
         <v>3888.32</v>
       </c>
@@ -6239,7 +6436,7 @@
         <v>7</v>
       </c>
       <c r="E28" s="5"/>
-      <c r="F28" s="86"/>
+      <c r="F28" s="68"/>
       <c r="G28" s="5">
         <v>3888.32</v>
       </c>
@@ -6378,17 +6575,16 @@
       <c r="A29" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B29" s="83" t="s">
+      <c r="B29" t="s">
         <v>75</v>
       </c>
-      <c r="C29" s="83">
+      <c r="C29">
         <v>12</v>
       </c>
-      <c r="D29" s="83">
+      <c r="D29">
         <v>8</v>
       </c>
-      <c r="E29" s="83"/>
-      <c r="F29" s="85"/>
+      <c r="F29" s="67"/>
       <c r="G29">
         <v>4309.7</v>
       </c>
@@ -6527,17 +6723,16 @@
       <c r="A30" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B30" s="83" t="s">
+      <c r="B30" t="s">
         <v>78</v>
       </c>
-      <c r="C30" s="83">
+      <c r="C30">
         <v>12</v>
       </c>
-      <c r="D30" s="83">
+      <c r="D30">
         <v>8</v>
       </c>
-      <c r="E30" s="83"/>
-      <c r="F30" s="85"/>
+      <c r="F30" s="67"/>
       <c r="G30">
         <v>4309.7</v>
       </c>
@@ -6676,17 +6871,16 @@
       <c r="A31" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B31" s="83" t="s">
+      <c r="B31" t="s">
         <v>78</v>
       </c>
-      <c r="C31" s="83">
+      <c r="C31">
         <v>12</v>
       </c>
-      <c r="D31" s="83">
+      <c r="D31">
         <v>8</v>
       </c>
-      <c r="E31" s="83"/>
-      <c r="F31" s="85"/>
+      <c r="F31" s="67"/>
       <c r="G31">
         <v>4309.7</v>
       </c>
@@ -6835,7 +7029,7 @@
         <v>9</v>
       </c>
       <c r="E32" s="3"/>
-      <c r="F32" s="84"/>
+      <c r="F32" s="66"/>
       <c r="G32" s="3">
         <v>4805.7299999999996</v>
       </c>
@@ -6974,17 +7168,16 @@
       <c r="A33" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B33" s="83" t="s">
+      <c r="B33" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="83">
+      <c r="C33">
         <v>12</v>
       </c>
-      <c r="D33" s="83">
+      <c r="D33">
         <v>9</v>
       </c>
-      <c r="E33" s="83"/>
-      <c r="F33" s="85"/>
+      <c r="F33" s="67"/>
       <c r="G33">
         <v>4805.7299999999996</v>
       </c>
@@ -7133,7 +7326,7 @@
         <v>9</v>
       </c>
       <c r="E34" s="5"/>
-      <c r="F34" s="86"/>
+      <c r="F34" s="68"/>
       <c r="G34" s="5">
         <v>4805.7299999999996</v>
       </c>
@@ -7272,17 +7465,16 @@
       <c r="A35" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="83" t="s">
+      <c r="B35" t="s">
         <v>75</v>
       </c>
-      <c r="C35" s="83">
+      <c r="C35">
         <v>12</v>
       </c>
-      <c r="D35" s="83">
+      <c r="D35">
         <v>10</v>
       </c>
-      <c r="E35" s="83"/>
-      <c r="F35" s="85"/>
+      <c r="F35" s="67"/>
       <c r="G35" s="62">
         <v>5497.99</v>
       </c>
@@ -7421,17 +7613,16 @@
       <c r="A36" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B36" s="83" t="s">
+      <c r="B36" t="s">
         <v>78</v>
       </c>
-      <c r="C36" s="83">
+      <c r="C36">
         <v>12</v>
       </c>
-      <c r="D36" s="83">
+      <c r="D36">
         <v>10</v>
       </c>
-      <c r="E36" s="83"/>
-      <c r="F36" s="85"/>
+      <c r="F36" s="67"/>
       <c r="G36" s="62">
         <v>5497.99</v>
       </c>
@@ -7570,17 +7761,16 @@
       <c r="A37" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B37" s="83" t="s">
+      <c r="B37" t="s">
         <v>78</v>
       </c>
-      <c r="C37" s="83">
+      <c r="C37">
         <v>12</v>
       </c>
-      <c r="D37" s="83">
+      <c r="D37">
         <v>10</v>
       </c>
-      <c r="E37" s="83"/>
-      <c r="F37" s="85"/>
+      <c r="F37" s="67"/>
       <c r="G37" s="62">
         <v>5497.99</v>
       </c>
@@ -7729,7 +7919,7 @@
         <v>11</v>
       </c>
       <c r="E38" s="3"/>
-      <c r="F38" s="84"/>
+      <c r="F38" s="66"/>
       <c r="G38" s="63">
         <v>6057.48</v>
       </c>
@@ -7868,17 +8058,16 @@
       <c r="A39" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B39" s="83" t="s">
+      <c r="B39" t="s">
         <v>78</v>
       </c>
-      <c r="C39" s="83">
+      <c r="C39">
         <v>12</v>
       </c>
-      <c r="D39" s="83">
+      <c r="D39">
         <v>11</v>
       </c>
-      <c r="E39" s="83"/>
-      <c r="F39" s="85"/>
+      <c r="F39" s="67"/>
       <c r="G39" s="62">
         <v>6057.48</v>
       </c>
@@ -8025,7 +8214,7 @@
         <v>11</v>
       </c>
       <c r="E40" s="5"/>
-      <c r="F40" s="86"/>
+      <c r="F40" s="68"/>
       <c r="G40" s="62">
         <v>6057.48</v>
       </c>
@@ -8173,7 +8362,7 @@
         <v>12</v>
       </c>
       <c r="E41" s="3"/>
-      <c r="F41" s="84"/>
+      <c r="F41" s="66"/>
       <c r="G41" s="63">
         <v>6478.05</v>
       </c>
@@ -8312,17 +8501,16 @@
       <c r="A42" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="83" t="s">
+      <c r="B42" t="s">
         <v>78</v>
       </c>
-      <c r="C42" s="83">
+      <c r="C42">
         <v>12</v>
       </c>
-      <c r="D42" s="83">
+      <c r="D42">
         <v>12</v>
       </c>
-      <c r="E42" s="83"/>
-      <c r="F42" s="85"/>
+      <c r="F42" s="67"/>
       <c r="G42" s="62">
         <v>6478.05</v>
       </c>
@@ -8470,7 +8658,7 @@
         <v>12</v>
       </c>
       <c r="E43" s="5"/>
-      <c r="F43" s="86"/>
+      <c r="F43" s="68"/>
       <c r="G43" s="64">
         <v>6478.05</v>
       </c>
@@ -8645,6 +8833,7 @@
   <ignoredErrors>
     <ignoredError sqref="BE8:BE10" formulaRange="1"/>
   </ignoredErrors>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -8659,15 +8848,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -8890,7 +9070,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
@@ -8908,15 +9088,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8935,13 +9116,27 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
     <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
MR24-038 D8: edited the data location in mpc_graphs_3L.py to plot MR24-038 data
</commit_message>
<xml_diff>
--- a/data/mr24-038-experiment/MR24-038-MasterDataTable.xlsx
+++ b/data/mr24-038-experiment/MR24-038-MasterDataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/MR24-038-MPC-3L/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="559" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{123E69FD-5553-4086-AA0E-C4845C436807}"/>
+  <xr:revisionPtr revIDLastSave="582" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A92E14B7-5C28-4C96-B3B1-B1EE03567F49}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
@@ -5692,7 +5692,7 @@
       </c>
       <c r="AM20" s="68">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>3.9685397916666663E-2</v>
       </c>
       <c r="AN20" s="67">
         <v>244</v>
@@ -5733,9 +5733,17 @@
       <c r="AY20" s="84">
         <v>4.0000000000000002E-4</v>
       </c>
-      <c r="AZ20" s="81"/>
-      <c r="BA20" s="69"/>
-      <c r="BB20" s="84"/>
+      <c r="AZ20" s="81">
+        <v>2.9899999999999999E-2</v>
+      </c>
+      <c r="BA20" s="99">
+        <f>BJ20*24*60/BE20</f>
+        <v>8.8711852715143927E-3</v>
+      </c>
+      <c r="BB20" s="99">
+        <f>BM20/BE20</f>
+        <v>9.9999999999999995E-8</v>
+      </c>
       <c r="BC20" s="81">
         <f t="shared" si="0"/>
         <v>1.80423888E-2</v>
@@ -5758,15 +5766,14 @@
       </c>
       <c r="BH20" s="70">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>57.146972999999988</v>
       </c>
       <c r="BI20" s="70">
         <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="BJ20" s="70" t="str">
-        <f t="shared" si="13"/>
-        <v/>
+        <v>3.9685397916666663E-2</v>
+      </c>
+      <c r="BJ20" s="70">
+        <v>1.1774465467977301E-2</v>
       </c>
       <c r="BK20" s="71" t="str">
         <f t="shared" si="6"/>
@@ -5776,17 +5783,16 @@
         <f t="shared" si="19"/>
         <v>0</v>
       </c>
-      <c r="BM20" s="82" t="str">
-        <f t="shared" si="14"/>
-        <v/>
+      <c r="BM20" s="82">
+        <v>1.91127E-4</v>
       </c>
       <c r="BN20" s="75">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>103.07895562770562</v>
       </c>
       <c r="BO20" s="72">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>3.9685397916666663E-2</v>
       </c>
       <c r="BP20" s="73">
         <f t="shared" si="7"/>
@@ -5812,57 +5818,119 @@
         <v>4309.7</v>
       </c>
       <c r="H21" s="67"/>
-      <c r="I21" s="67"/>
-      <c r="J21" s="67"/>
-      <c r="K21" s="67"/>
-      <c r="L21" s="67"/>
-      <c r="M21" s="67"/>
-      <c r="N21" s="67"/>
-      <c r="O21" s="67"/>
-      <c r="P21" s="67"/>
-      <c r="Q21" s="67"/>
+      <c r="I21" s="67">
+        <v>4097.625</v>
+      </c>
+      <c r="J21" s="67">
+        <v>25.3</v>
+      </c>
+      <c r="K21" s="67">
+        <v>24</v>
+      </c>
+      <c r="L21" s="67">
+        <v>94.8</v>
+      </c>
+      <c r="M21" s="67">
+        <v>18.8</v>
+      </c>
+      <c r="N21" s="67">
+        <v>458</v>
+      </c>
+      <c r="O21" s="67">
+        <v>3</v>
+      </c>
+      <c r="P21" s="67">
+        <v>0.25</v>
+      </c>
+      <c r="Q21" s="67">
+        <v>7.34</v>
+      </c>
       <c r="R21" s="67"/>
-      <c r="S21" s="67"/>
-      <c r="T21" s="67"/>
-      <c r="U21" s="67"/>
-      <c r="V21" s="67"/>
-      <c r="W21" s="67"/>
-      <c r="X21" s="67"/>
-      <c r="Y21" s="67"/>
-      <c r="Z21" s="67"/>
-      <c r="AA21" s="67"/>
-      <c r="AB21" s="67"/>
-      <c r="AC21" s="67"/>
-      <c r="AD21" s="96"/>
-      <c r="AE21" s="91"/>
-      <c r="AF21" s="67"/>
-      <c r="AG21" s="67"/>
+      <c r="S21" s="67">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="T21" s="67">
+        <v>3.94</v>
+      </c>
+      <c r="U21" s="67">
+        <v>1.89</v>
+      </c>
+      <c r="V21" s="67">
+        <v>7.0620000000000003</v>
+      </c>
+      <c r="W21" s="67">
+        <v>165.6</v>
+      </c>
+      <c r="X21" s="67">
+        <v>9</v>
+      </c>
+      <c r="Y21" s="67">
+        <v>1.51</v>
+      </c>
+      <c r="Z21" s="67">
+        <v>165.7</v>
+      </c>
+      <c r="AA21" s="67">
+        <v>45.5</v>
+      </c>
+      <c r="AB21" s="67">
+        <v>145.19999999999999</v>
+      </c>
+      <c r="AC21" s="67">
+        <v>7.3</v>
+      </c>
+      <c r="AD21" s="96">
+        <v>7.1</v>
+      </c>
+      <c r="AE21" s="91">
+        <v>300</v>
+      </c>
+      <c r="AF21" s="67">
+        <v>49.9</v>
+      </c>
+      <c r="AG21" s="67">
+        <v>7.1</v>
+      </c>
       <c r="AH21" s="68">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="AI21" s="67"/>
-      <c r="AJ21" s="67"/>
-      <c r="AK21" s="67"/>
-      <c r="AL21" s="67"/>
+        <v>0.499</v>
+      </c>
+      <c r="AI21" s="67">
+        <v>34</v>
+      </c>
+      <c r="AJ21" s="67">
+        <v>32.640999999999998</v>
+      </c>
+      <c r="AK21" s="67">
+        <v>8.1745999999999999</v>
+      </c>
+      <c r="AL21" s="67">
+        <v>7</v>
+      </c>
       <c r="AM21" s="68">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="AN21" s="67"/>
-      <c r="AO21" s="67"/>
-      <c r="AP21" s="67"/>
+      <c r="AN21" s="67">
+        <v>303</v>
+      </c>
+      <c r="AO21" s="67">
+        <v>43</v>
+      </c>
+      <c r="AP21" s="67">
+        <v>387</v>
+      </c>
       <c r="AQ21" s="68">
         <f t="shared" si="24"/>
-        <v>-244</v>
+        <v>59</v>
       </c>
       <c r="AR21" s="68">
         <f t="shared" si="24"/>
-        <v>-43</v>
+        <v>0</v>
       </c>
       <c r="AS21" s="68">
         <f t="shared" si="25"/>
-        <v>450</v>
+        <v>63</v>
       </c>
       <c r="AT21" s="92">
         <v>15</v>
@@ -5887,23 +5955,23 @@
       <c r="BB21" s="84"/>
       <c r="BC21" s="81">
         <f t="shared" ref="BC21:BC25" si="26">AY21*K21*BE21/1000</f>
-        <v>0</v>
+        <v>1.880462976E-2</v>
       </c>
       <c r="BD21" s="69">
         <f t="shared" ref="BD21:BD25" si="27">BC21*24*60</f>
-        <v>0</v>
+        <v>27.078666854400002</v>
       </c>
       <c r="BE21" s="69">
         <f t="shared" si="17"/>
-        <v>1565</v>
-      </c>
-      <c r="BF21" s="70" t="e">
+        <v>1958.8155999999999</v>
+      </c>
+      <c r="BF21" s="70">
         <f t="shared" ref="BF21:BF25" si="28">IF(ISBLANK(AN21),NA(),IFERROR(AN21/BE21,0))</f>
-        <v>#N/A</v>
-      </c>
-      <c r="BG21" s="70" t="e">
+        <v>0.15468531085825538</v>
+      </c>
+      <c r="BG21" s="70">
         <f t="shared" ref="BG21:BG25" si="29">IF(ISBLANK(AN21),NA(),AN21/AU21)</f>
-        <v>#N/A</v>
+        <v>0.17823529411764705</v>
       </c>
       <c r="BH21" s="70">
         <f t="shared" ref="BH21:BH25" si="30">AM21*24*60</f>
@@ -5923,7 +5991,7 @@
       </c>
       <c r="BL21" s="70">
         <f t="shared" si="19"/>
-        <v>11.737500000000001</v>
+        <v>0</v>
       </c>
       <c r="BM21" s="82" t="str">
         <f t="shared" si="14"/>
@@ -5939,7 +6007,7 @@
       </c>
       <c r="BP21" s="73">
         <f t="shared" ref="BP21:BP25" si="32">IF(BL21&lt;&gt;"",BL21,BM21)</f>
-        <v>11.737500000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:68" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6003,15 +6071,15 @@
       <c r="AP22" s="67"/>
       <c r="AQ22" s="68">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>-303</v>
       </c>
       <c r="AR22" s="68">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>-43</v>
       </c>
       <c r="AS22" s="68">
         <f t="shared" si="25"/>
-        <v>0</v>
+        <v>387</v>
       </c>
       <c r="AT22" s="92">
         <v>15</v>
@@ -6847,14 +6915,14 @@
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>